<commit_message>
Add LTV-dilution handling for 1-mo trial (realization lever + sensitivity + breakeven)
Addresses lead feedback that LTV may drop with a 1-month trial (marginal-
converter dilution). Adds an adjustable 'LTV realization factor' (Assumptions
B19, default 100%) applied to go-forward 1-mo-era LTV, a new LTV sensitivity
tab (LTV:CAC & net contribution across 130%->60% of observed) and a breakeven
block (breakeven LTV = payout; $350 needs ~2.13x observed LTV). Conclusion is
robust across the full haircut range.

Co-authored-by: johnkalis <johnkalis@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/analysis/adrian-morrison/adrian_morrison_1mo_trial_icac_ltv.xlsx
+++ b/analysis/adrian-morrison/adrian_morrison_1mo_trial_icac_ltv.xlsx
@@ -10,7 +10,8 @@
     <sheet name="Assumptions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Scenarios" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="IAF sensitivity" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="README" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="LTV sensitivity" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="README" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -141,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -177,6 +178,9 @@
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -286,6 +290,27 @@
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -656,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -931,43 +956,58 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>IAF sensitivity — low</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="n">
-        <v>0.38</v>
+          <t>LTV realization factor (go-forward)</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Current incrementality.</t>
+          <t>STRESS-TEST LEVER for the lead's 'LTV drops with a 1-mo trial' concern. % of observed 1-mo-era LTV assumed to hold. The observed number already includes marginal (lower-intent) converters, so 100% = no extra haircut; lower it (e.g. 80%) to be conservative for marginal-converter dilution / forecast risk.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>IAF sensitivity — mid</t>
+          <t>IAF sensitivity — low</t>
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>0.6</v>
+        <v>0.38</v>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>If a fresh 1-mo funnel re-baselines incrementality.</t>
+          <t>Current incrementality.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
+          <t>IAF sensitivity — mid</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>If a fresh 1-mo funnel re-baselines incrementality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
           <t>IAF sensitivity — high</t>
         </is>
       </c>
-      <c r="B21" s="9" t="n">
+      <c r="B22" s="9" t="n">
         <v>0.75</v>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>Upper incrementality scenario.</t>
         </is>
@@ -987,7 +1027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W15"/>
+  <dimension ref="A1:W16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1045,876 +1085,883 @@
       <c r="W1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>SCENARIO</t>
         </is>
       </c>
-      <c r="B2" s="14" t="n"/>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="15" t="inlineStr">
+      <c r="B2" s="15" t="n"/>
+      <c r="C2" s="15" t="n"/>
+      <c r="D2" s="15" t="n"/>
+      <c r="E2" s="15" t="n"/>
+      <c r="F2" s="16" t="inlineStr">
         <is>
           <t>WHAT WE GET</t>
         </is>
       </c>
-      <c r="G2" s="16" t="n"/>
-      <c r="H2" s="16" t="n"/>
-      <c r="I2" s="17" t="inlineStr">
+      <c r="G2" s="17" t="n"/>
+      <c r="H2" s="17" t="n"/>
+      <c r="I2" s="18" t="inlineStr">
         <is>
           <t>WHAT IT COSTS</t>
         </is>
       </c>
-      <c r="J2" s="18" t="n"/>
-      <c r="K2" s="18" t="n"/>
-      <c r="L2" s="18" t="n"/>
-      <c r="M2" s="18" t="n"/>
-      <c r="N2" s="19" t="inlineStr">
+      <c r="J2" s="19" t="n"/>
+      <c r="K2" s="19" t="n"/>
+      <c r="L2" s="19" t="n"/>
+      <c r="M2" s="19" t="n"/>
+      <c r="N2" s="20" t="inlineStr">
         <is>
           <t>LTV PER SHOP  &amp;  LTV:CAC</t>
         </is>
       </c>
-      <c r="O2" s="20" t="n"/>
-      <c r="P2" s="20" t="n"/>
-      <c r="Q2" s="20" t="n"/>
-      <c r="R2" s="20" t="n"/>
-      <c r="S2" s="20" t="n"/>
-      <c r="T2" s="21" t="inlineStr">
+      <c r="O2" s="21" t="n"/>
+      <c r="P2" s="21" t="n"/>
+      <c r="Q2" s="21" t="n"/>
+      <c r="R2" s="21" t="n"/>
+      <c r="S2" s="21" t="n"/>
+      <c r="T2" s="22" t="inlineStr">
         <is>
           <t>TOTALS &amp; RETURNS</t>
         </is>
       </c>
-      <c r="U2" s="22" t="n"/>
-      <c r="V2" s="22" t="n"/>
-      <c r="W2" s="22" t="n"/>
+      <c r="U2" s="23" t="n"/>
+      <c r="V2" s="23" t="n"/>
+      <c r="W2" s="23" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="inlineStr">
+      <c r="A3" s="24" t="inlineStr">
         <is>
           <t>Scenario</t>
         </is>
       </c>
-      <c r="B3" s="23" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Trial era</t>
         </is>
       </c>
-      <c r="C3" s="23" t="inlineStr">
+      <c r="C3" s="24" t="inlineStr">
         <is>
           <t>Paid trials / mo</t>
         </is>
       </c>
-      <c r="D3" s="23" t="inlineStr">
+      <c r="D3" s="24" t="inlineStr">
         <is>
           <t>Payout ($)</t>
         </is>
       </c>
-      <c r="E3" s="23" t="inlineStr">
+      <c r="E3" s="24" t="inlineStr">
         <is>
           <t>Payout basis</t>
         </is>
       </c>
-      <c r="F3" s="23" t="inlineStr">
+      <c r="F3" s="24" t="inlineStr">
         <is>
           <t>Trial→FP CVR</t>
         </is>
       </c>
-      <c r="G3" s="23" t="inlineStr">
+      <c r="G3" s="24" t="inlineStr">
         <is>
           <t>FP shops / mo</t>
         </is>
       </c>
-      <c r="H3" s="23" t="inlineStr">
+      <c r="H3" s="24" t="inlineStr">
         <is>
           <t>iGA / mo</t>
         </is>
       </c>
-      <c r="I3" s="23" t="inlineStr">
+      <c r="I3" s="24" t="inlineStr">
         <is>
           <t>Monthly spend</t>
         </is>
       </c>
-      <c r="J3" s="23" t="inlineStr">
+      <c r="J3" s="24" t="inlineStr">
         <is>
           <t>Annual spend</t>
         </is>
       </c>
-      <c r="K3" s="23" t="inlineStr">
+      <c r="K3" s="24" t="inlineStr">
         <is>
           <t>Cost / FP shop</t>
         </is>
       </c>
-      <c r="L3" s="23" t="inlineStr">
+      <c r="L3" s="24" t="inlineStr">
         <is>
           <t>iCAC</t>
         </is>
       </c>
-      <c r="M3" s="23" t="inlineStr">
+      <c r="M3" s="24" t="inlineStr">
         <is>
           <t>iCAC vs $267</t>
         </is>
       </c>
-      <c r="N3" s="23" t="inlineStr">
+      <c r="N3" s="24" t="inlineStr">
         <is>
           <t>LTV/shop @12mo</t>
         </is>
       </c>
-      <c r="O3" s="23" t="inlineStr">
+      <c r="O3" s="24" t="inlineStr">
         <is>
           <t>LTV/shop @24mo</t>
         </is>
       </c>
-      <c r="P3" s="23" t="inlineStr">
+      <c r="P3" s="24" t="inlineStr">
         <is>
           <t>LTV/shop @36mo</t>
         </is>
       </c>
-      <c r="Q3" s="23" t="inlineStr">
+      <c r="Q3" s="24" t="inlineStr">
         <is>
           <t>LTV:CAC @12mo</t>
         </is>
       </c>
-      <c r="R3" s="23" t="inlineStr">
+      <c r="R3" s="24" t="inlineStr">
         <is>
           <t>LTV:CAC @24mo</t>
         </is>
       </c>
-      <c r="S3" s="23" t="inlineStr">
+      <c r="S3" s="24" t="inlineStr">
         <is>
           <t>LTV:CAC @36mo</t>
         </is>
       </c>
-      <c r="T3" s="23" t="inlineStr">
+      <c r="T3" s="24" t="inlineStr">
         <is>
           <t>Total LTV/mo @36mo</t>
         </is>
       </c>
-      <c r="U3" s="23" t="inlineStr">
+      <c r="U3" s="24" t="inlineStr">
         <is>
           <t>Total LTV/yr @36mo</t>
         </is>
       </c>
-      <c r="V3" s="23" t="inlineStr">
+      <c r="V3" s="24" t="inlineStr">
         <is>
           <t>Net contrib/shop @36mo</t>
         </is>
       </c>
-      <c r="W3" s="23" t="inlineStr">
+      <c r="W3" s="24" t="inlineStr">
         <is>
           <t>Net contrib/yr @36mo</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>Current (3-mo @ $90)</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="26" t="inlineStr">
         <is>
           <t>3-mo</t>
         </is>
       </c>
-      <c r="C4" s="26">
+      <c r="C4" s="27">
         <f>Assumptions!$B$3</f>
         <v/>
       </c>
-      <c r="D4" s="27">
+      <c r="D4" s="28">
         <f>Assumptions!$B$9</f>
         <v/>
       </c>
-      <c r="E4" s="25" t="inlineStr">
+      <c r="E4" s="26" t="inlineStr">
         <is>
           <t>per paid trial</t>
         </is>
       </c>
-      <c r="F4" s="28">
+      <c r="F4" s="29">
         <f>Assumptions!$B$6</f>
         <v/>
       </c>
-      <c r="G4" s="26">
+      <c r="G4" s="27">
         <f>C4*F4</f>
         <v/>
       </c>
-      <c r="H4" s="26">
+      <c r="H4" s="27">
         <f>C4*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="I4" s="27">
+      <c r="I4" s="28">
         <f>D4*C4</f>
         <v/>
       </c>
-      <c r="J4" s="27">
+      <c r="J4" s="28">
         <f>I4*12</f>
         <v/>
       </c>
-      <c r="K4" s="27">
+      <c r="K4" s="28">
         <f>I4/G4</f>
         <v/>
       </c>
-      <c r="L4" s="29">
+      <c r="L4" s="30">
         <f>I4/H4</f>
         <v/>
       </c>
-      <c r="M4" s="30">
+      <c r="M4" s="31">
         <f>L4/Assumptions!$B$8-1</f>
         <v/>
       </c>
-      <c r="N4" s="31">
+      <c r="N4" s="32">
         <f>Assumptions!$B$16</f>
         <v/>
       </c>
-      <c r="O4" s="31">
+      <c r="O4" s="32">
         <f>Assumptions!$B$17</f>
         <v/>
       </c>
-      <c r="P4" s="31">
+      <c r="P4" s="32">
         <f>IF(Assumptions!$B$18="","n.a.",Assumptions!$B$18)</f>
         <v/>
       </c>
-      <c r="Q4" s="32">
+      <c r="Q4" s="33">
         <f>N4/K4</f>
         <v/>
       </c>
-      <c r="R4" s="32">
+      <c r="R4" s="33">
         <f>O4/K4</f>
         <v/>
       </c>
-      <c r="S4" s="33">
+      <c r="S4" s="34">
         <f>IF(Assumptions!$B$18="","n.a.",Assumptions!$B$18/K4)</f>
         <v/>
       </c>
-      <c r="T4" s="27">
+      <c r="T4" s="28">
         <f>IF(Assumptions!$B$18="","n.a.",Assumptions!$B$18*G4)</f>
         <v/>
       </c>
-      <c r="U4" s="27">
+      <c r="U4" s="28">
         <f>IF(Assumptions!$B$18="","n.a.",Assumptions!$B$18*G4*12)</f>
         <v/>
       </c>
-      <c r="V4" s="34">
+      <c r="V4" s="35">
         <f>IF(Assumptions!$B$18="","n.a.",Assumptions!$B$18-K4)</f>
         <v/>
       </c>
-      <c r="W4" s="35">
+      <c r="W4" s="36">
         <f>IF(Assumptions!$B$18="","n.a.",(Assumptions!$B$18-K4)*G4*12)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="36" t="inlineStr">
+      <c r="A5" s="37" t="inlineStr">
         <is>
           <t>$250 / FP · base 8.9k</t>
         </is>
       </c>
-      <c r="B5" s="37" t="inlineStr">
+      <c r="B5" s="38" t="inlineStr">
         <is>
           <t>1-mo</t>
         </is>
       </c>
-      <c r="C5" s="38">
+      <c r="C5" s="39">
         <f>Assumptions!$B$3</f>
         <v/>
       </c>
-      <c r="D5" s="39">
+      <c r="D5" s="40">
         <f>Assumptions!$B$10</f>
         <v/>
       </c>
-      <c r="E5" s="37" t="inlineStr">
+      <c r="E5" s="38" t="inlineStr">
         <is>
           <t>per FP conv.</t>
         </is>
       </c>
-      <c r="F5" s="40">
+      <c r="F5" s="41">
         <f>Assumptions!$B$5</f>
         <v/>
       </c>
-      <c r="G5" s="38">
+      <c r="G5" s="39">
         <f>C5*F5</f>
         <v/>
       </c>
-      <c r="H5" s="38">
+      <c r="H5" s="39">
         <f>C5*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="I5" s="39">
+      <c r="I5" s="40">
         <f>D5*G5</f>
         <v/>
       </c>
-      <c r="J5" s="39">
+      <c r="J5" s="40">
         <f>I5*12</f>
         <v/>
       </c>
-      <c r="K5" s="39">
+      <c r="K5" s="40">
         <f>I5/G5</f>
         <v/>
       </c>
-      <c r="L5" s="41">
+      <c r="L5" s="42">
         <f>I5/H5</f>
         <v/>
       </c>
-      <c r="M5" s="42">
+      <c r="M5" s="43">
         <f>L5/Assumptions!$B$8-1</f>
         <v/>
       </c>
-      <c r="N5" s="43">
-        <f>Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="O5" s="43">
-        <f>Assumptions!$B$14</f>
-        <v/>
-      </c>
-      <c r="P5" s="43">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15)</f>
-        <v/>
-      </c>
-      <c r="Q5" s="44">
+      <c r="N5" s="44">
+        <f>Assumptions!$B$13*Assumptions!$B$19</f>
+        <v/>
+      </c>
+      <c r="O5" s="44">
+        <f>Assumptions!$B$14*Assumptions!$B$19</f>
+        <v/>
+      </c>
+      <c r="P5" s="44">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19)</f>
+        <v/>
+      </c>
+      <c r="Q5" s="45">
         <f>N5/K5</f>
         <v/>
       </c>
-      <c r="R5" s="44">
+      <c r="R5" s="45">
         <f>O5/K5</f>
         <v/>
       </c>
-      <c r="S5" s="45">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15/K5)</f>
-        <v/>
-      </c>
-      <c r="T5" s="39">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*G5)</f>
-        <v/>
-      </c>
-      <c r="U5" s="39">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*G5*12)</f>
-        <v/>
-      </c>
-      <c r="V5" s="46">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15-K5)</f>
-        <v/>
-      </c>
-      <c r="W5" s="47">
-        <f>IF(Assumptions!$B$15="","n.a.",(Assumptions!$B$15-K5)*G5*12)</f>
+      <c r="S5" s="46">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19/K5)</f>
+        <v/>
+      </c>
+      <c r="T5" s="40">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19*G5)</f>
+        <v/>
+      </c>
+      <c r="U5" s="40">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19*G5*12)</f>
+        <v/>
+      </c>
+      <c r="V5" s="47">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19-K5)</f>
+        <v/>
+      </c>
+      <c r="W5" s="48">
+        <f>IF(Assumptions!$B$15="","n.a.",(Assumptions!$B$15*Assumptions!$B$19-K5)*G5*12)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="36" t="inlineStr">
+      <c r="A6" s="37" t="inlineStr">
         <is>
           <t>$300 / FP · base 8.9k</t>
         </is>
       </c>
-      <c r="B6" s="37" t="inlineStr">
+      <c r="B6" s="38" t="inlineStr">
         <is>
           <t>1-mo</t>
         </is>
       </c>
-      <c r="C6" s="38">
+      <c r="C6" s="39">
         <f>Assumptions!$B$3</f>
         <v/>
       </c>
-      <c r="D6" s="39">
+      <c r="D6" s="40">
         <f>Assumptions!$B$11</f>
         <v/>
       </c>
-      <c r="E6" s="37" t="inlineStr">
+      <c r="E6" s="38" t="inlineStr">
         <is>
           <t>per FP conv.</t>
         </is>
       </c>
-      <c r="F6" s="40">
+      <c r="F6" s="41">
         <f>Assumptions!$B$5</f>
         <v/>
       </c>
-      <c r="G6" s="38">
+      <c r="G6" s="39">
         <f>C6*F6</f>
         <v/>
       </c>
-      <c r="H6" s="38">
+      <c r="H6" s="39">
         <f>C6*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="I6" s="39">
+      <c r="I6" s="40">
         <f>D6*G6</f>
         <v/>
       </c>
-      <c r="J6" s="39">
+      <c r="J6" s="40">
         <f>I6*12</f>
         <v/>
       </c>
-      <c r="K6" s="39">
+      <c r="K6" s="40">
         <f>I6/G6</f>
         <v/>
       </c>
-      <c r="L6" s="41">
+      <c r="L6" s="42">
         <f>I6/H6</f>
         <v/>
       </c>
-      <c r="M6" s="42">
+      <c r="M6" s="43">
         <f>L6/Assumptions!$B$8-1</f>
         <v/>
       </c>
-      <c r="N6" s="43">
-        <f>Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="O6" s="43">
-        <f>Assumptions!$B$14</f>
-        <v/>
-      </c>
-      <c r="P6" s="43">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15)</f>
-        <v/>
-      </c>
-      <c r="Q6" s="44">
+      <c r="N6" s="44">
+        <f>Assumptions!$B$13*Assumptions!$B$19</f>
+        <v/>
+      </c>
+      <c r="O6" s="44">
+        <f>Assumptions!$B$14*Assumptions!$B$19</f>
+        <v/>
+      </c>
+      <c r="P6" s="44">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19)</f>
+        <v/>
+      </c>
+      <c r="Q6" s="45">
         <f>N6/K6</f>
         <v/>
       </c>
-      <c r="R6" s="44">
+      <c r="R6" s="45">
         <f>O6/K6</f>
         <v/>
       </c>
-      <c r="S6" s="45">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15/K6)</f>
-        <v/>
-      </c>
-      <c r="T6" s="39">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*G6)</f>
-        <v/>
-      </c>
-      <c r="U6" s="39">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*G6*12)</f>
-        <v/>
-      </c>
-      <c r="V6" s="46">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15-K6)</f>
-        <v/>
-      </c>
-      <c r="W6" s="47">
-        <f>IF(Assumptions!$B$15="","n.a.",(Assumptions!$B$15-K6)*G6*12)</f>
+      <c r="S6" s="46">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19/K6)</f>
+        <v/>
+      </c>
+      <c r="T6" s="40">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19*G6)</f>
+        <v/>
+      </c>
+      <c r="U6" s="40">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19*G6*12)</f>
+        <v/>
+      </c>
+      <c r="V6" s="47">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19-K6)</f>
+        <v/>
+      </c>
+      <c r="W6" s="48">
+        <f>IF(Assumptions!$B$15="","n.a.",(Assumptions!$B$15*Assumptions!$B$19-K6)*G6*12)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="36" t="inlineStr">
+      <c r="A7" s="37" t="inlineStr">
         <is>
           <t>$350 / FP · base 8.9k</t>
         </is>
       </c>
-      <c r="B7" s="37" t="inlineStr">
+      <c r="B7" s="38" t="inlineStr">
         <is>
           <t>1-mo</t>
         </is>
       </c>
-      <c r="C7" s="38">
+      <c r="C7" s="39">
         <f>Assumptions!$B$3</f>
         <v/>
       </c>
-      <c r="D7" s="39">
+      <c r="D7" s="40">
         <f>Assumptions!$B$12</f>
         <v/>
       </c>
-      <c r="E7" s="37" t="inlineStr">
+      <c r="E7" s="38" t="inlineStr">
         <is>
           <t>per FP conv.</t>
         </is>
       </c>
-      <c r="F7" s="40">
+      <c r="F7" s="41">
         <f>Assumptions!$B$5</f>
         <v/>
       </c>
-      <c r="G7" s="38">
+      <c r="G7" s="39">
         <f>C7*F7</f>
         <v/>
       </c>
-      <c r="H7" s="38">
+      <c r="H7" s="39">
         <f>C7*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="I7" s="39">
+      <c r="I7" s="40">
         <f>D7*G7</f>
         <v/>
       </c>
-      <c r="J7" s="39">
+      <c r="J7" s="40">
         <f>I7*12</f>
         <v/>
       </c>
-      <c r="K7" s="39">
+      <c r="K7" s="40">
         <f>I7/G7</f>
         <v/>
       </c>
-      <c r="L7" s="41">
+      <c r="L7" s="42">
         <f>I7/H7</f>
         <v/>
       </c>
-      <c r="M7" s="42">
+      <c r="M7" s="43">
         <f>L7/Assumptions!$B$8-1</f>
         <v/>
       </c>
-      <c r="N7" s="43">
-        <f>Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="O7" s="43">
-        <f>Assumptions!$B$14</f>
-        <v/>
-      </c>
-      <c r="P7" s="43">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15)</f>
-        <v/>
-      </c>
-      <c r="Q7" s="44">
+      <c r="N7" s="44">
+        <f>Assumptions!$B$13*Assumptions!$B$19</f>
+        <v/>
+      </c>
+      <c r="O7" s="44">
+        <f>Assumptions!$B$14*Assumptions!$B$19</f>
+        <v/>
+      </c>
+      <c r="P7" s="44">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19)</f>
+        <v/>
+      </c>
+      <c r="Q7" s="45">
         <f>N7/K7</f>
         <v/>
       </c>
-      <c r="R7" s="44">
+      <c r="R7" s="45">
         <f>O7/K7</f>
         <v/>
       </c>
-      <c r="S7" s="45">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15/K7)</f>
-        <v/>
-      </c>
-      <c r="T7" s="39">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*G7)</f>
-        <v/>
-      </c>
-      <c r="U7" s="39">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*G7*12)</f>
-        <v/>
-      </c>
-      <c r="V7" s="46">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15-K7)</f>
-        <v/>
-      </c>
-      <c r="W7" s="47">
-        <f>IF(Assumptions!$B$15="","n.a.",(Assumptions!$B$15-K7)*G7*12)</f>
+      <c r="S7" s="46">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19/K7)</f>
+        <v/>
+      </c>
+      <c r="T7" s="40">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19*G7)</f>
+        <v/>
+      </c>
+      <c r="U7" s="40">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19*G7*12)</f>
+        <v/>
+      </c>
+      <c r="V7" s="47">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19-K7)</f>
+        <v/>
+      </c>
+      <c r="W7" s="48">
+        <f>IF(Assumptions!$B$15="","n.a.",(Assumptions!$B$15*Assumptions!$B$19-K7)*G7*12)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="36" t="inlineStr">
+      <c r="A8" s="37" t="inlineStr">
         <is>
           <t>$250 / FP · stretch 12k</t>
         </is>
       </c>
-      <c r="B8" s="37" t="inlineStr">
+      <c r="B8" s="38" t="inlineStr">
         <is>
           <t>1-mo</t>
         </is>
       </c>
-      <c r="C8" s="38">
+      <c r="C8" s="39">
         <f>Assumptions!$B$4</f>
         <v/>
       </c>
-      <c r="D8" s="39">
+      <c r="D8" s="40">
         <f>Assumptions!$B$10</f>
         <v/>
       </c>
-      <c r="E8" s="37" t="inlineStr">
+      <c r="E8" s="38" t="inlineStr">
         <is>
           <t>per FP conv.</t>
         </is>
       </c>
-      <c r="F8" s="40">
+      <c r="F8" s="41">
         <f>Assumptions!$B$5</f>
         <v/>
       </c>
-      <c r="G8" s="38">
+      <c r="G8" s="39">
         <f>C8*F8</f>
         <v/>
       </c>
-      <c r="H8" s="38">
+      <c r="H8" s="39">
         <f>C8*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="I8" s="39">
+      <c r="I8" s="40">
         <f>D8*G8</f>
         <v/>
       </c>
-      <c r="J8" s="39">
+      <c r="J8" s="40">
         <f>I8*12</f>
         <v/>
       </c>
-      <c r="K8" s="39">
+      <c r="K8" s="40">
         <f>I8/G8</f>
         <v/>
       </c>
-      <c r="L8" s="41">
+      <c r="L8" s="42">
         <f>I8/H8</f>
         <v/>
       </c>
-      <c r="M8" s="42">
+      <c r="M8" s="43">
         <f>L8/Assumptions!$B$8-1</f>
         <v/>
       </c>
-      <c r="N8" s="43">
-        <f>Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="O8" s="43">
-        <f>Assumptions!$B$14</f>
-        <v/>
-      </c>
-      <c r="P8" s="43">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15)</f>
-        <v/>
-      </c>
-      <c r="Q8" s="44">
+      <c r="N8" s="44">
+        <f>Assumptions!$B$13*Assumptions!$B$19</f>
+        <v/>
+      </c>
+      <c r="O8" s="44">
+        <f>Assumptions!$B$14*Assumptions!$B$19</f>
+        <v/>
+      </c>
+      <c r="P8" s="44">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="45">
         <f>N8/K8</f>
         <v/>
       </c>
-      <c r="R8" s="44">
+      <c r="R8" s="45">
         <f>O8/K8</f>
         <v/>
       </c>
-      <c r="S8" s="45">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15/K8)</f>
-        <v/>
-      </c>
-      <c r="T8" s="39">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*G8)</f>
-        <v/>
-      </c>
-      <c r="U8" s="39">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*G8*12)</f>
-        <v/>
-      </c>
-      <c r="V8" s="46">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15-K8)</f>
-        <v/>
-      </c>
-      <c r="W8" s="47">
-        <f>IF(Assumptions!$B$15="","n.a.",(Assumptions!$B$15-K8)*G8*12)</f>
+      <c r="S8" s="46">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19/K8)</f>
+        <v/>
+      </c>
+      <c r="T8" s="40">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19*G8)</f>
+        <v/>
+      </c>
+      <c r="U8" s="40">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19*G8*12)</f>
+        <v/>
+      </c>
+      <c r="V8" s="47">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19-K8)</f>
+        <v/>
+      </c>
+      <c r="W8" s="48">
+        <f>IF(Assumptions!$B$15="","n.a.",(Assumptions!$B$15*Assumptions!$B$19-K8)*G8*12)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="36" t="inlineStr">
+      <c r="A9" s="37" t="inlineStr">
         <is>
           <t>$300 / FP · stretch 12k</t>
         </is>
       </c>
-      <c r="B9" s="37" t="inlineStr">
+      <c r="B9" s="38" t="inlineStr">
         <is>
           <t>1-mo</t>
         </is>
       </c>
-      <c r="C9" s="38">
+      <c r="C9" s="39">
         <f>Assumptions!$B$4</f>
         <v/>
       </c>
-      <c r="D9" s="39">
+      <c r="D9" s="40">
         <f>Assumptions!$B$11</f>
         <v/>
       </c>
-      <c r="E9" s="37" t="inlineStr">
+      <c r="E9" s="38" t="inlineStr">
         <is>
           <t>per FP conv.</t>
         </is>
       </c>
-      <c r="F9" s="40">
+      <c r="F9" s="41">
         <f>Assumptions!$B$5</f>
         <v/>
       </c>
-      <c r="G9" s="38">
+      <c r="G9" s="39">
         <f>C9*F9</f>
         <v/>
       </c>
-      <c r="H9" s="38">
+      <c r="H9" s="39">
         <f>C9*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="I9" s="39">
+      <c r="I9" s="40">
         <f>D9*G9</f>
         <v/>
       </c>
-      <c r="J9" s="39">
+      <c r="J9" s="40">
         <f>I9*12</f>
         <v/>
       </c>
-      <c r="K9" s="39">
+      <c r="K9" s="40">
         <f>I9/G9</f>
         <v/>
       </c>
-      <c r="L9" s="41">
+      <c r="L9" s="42">
         <f>I9/H9</f>
         <v/>
       </c>
-      <c r="M9" s="42">
+      <c r="M9" s="43">
         <f>L9/Assumptions!$B$8-1</f>
         <v/>
       </c>
-      <c r="N9" s="43">
-        <f>Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="O9" s="43">
-        <f>Assumptions!$B$14</f>
-        <v/>
-      </c>
-      <c r="P9" s="43">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15)</f>
-        <v/>
-      </c>
-      <c r="Q9" s="44">
+      <c r="N9" s="44">
+        <f>Assumptions!$B$13*Assumptions!$B$19</f>
+        <v/>
+      </c>
+      <c r="O9" s="44">
+        <f>Assumptions!$B$14*Assumptions!$B$19</f>
+        <v/>
+      </c>
+      <c r="P9" s="44">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="45">
         <f>N9/K9</f>
         <v/>
       </c>
-      <c r="R9" s="44">
+      <c r="R9" s="45">
         <f>O9/K9</f>
         <v/>
       </c>
-      <c r="S9" s="45">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15/K9)</f>
-        <v/>
-      </c>
-      <c r="T9" s="39">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*G9)</f>
-        <v/>
-      </c>
-      <c r="U9" s="39">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*G9*12)</f>
-        <v/>
-      </c>
-      <c r="V9" s="46">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15-K9)</f>
-        <v/>
-      </c>
-      <c r="W9" s="47">
-        <f>IF(Assumptions!$B$15="","n.a.",(Assumptions!$B$15-K9)*G9*12)</f>
+      <c r="S9" s="46">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19/K9)</f>
+        <v/>
+      </c>
+      <c r="T9" s="40">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19*G9)</f>
+        <v/>
+      </c>
+      <c r="U9" s="40">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19*G9*12)</f>
+        <v/>
+      </c>
+      <c r="V9" s="47">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19-K9)</f>
+        <v/>
+      </c>
+      <c r="W9" s="48">
+        <f>IF(Assumptions!$B$15="","n.a.",(Assumptions!$B$15*Assumptions!$B$19-K9)*G9*12)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="36" t="inlineStr">
+      <c r="A10" s="37" t="inlineStr">
         <is>
           <t>$350 / FP · stretch 12k</t>
         </is>
       </c>
-      <c r="B10" s="37" t="inlineStr">
+      <c r="B10" s="38" t="inlineStr">
         <is>
           <t>1-mo</t>
         </is>
       </c>
-      <c r="C10" s="38">
+      <c r="C10" s="39">
         <f>Assumptions!$B$4</f>
         <v/>
       </c>
-      <c r="D10" s="39">
+      <c r="D10" s="40">
         <f>Assumptions!$B$12</f>
         <v/>
       </c>
-      <c r="E10" s="37" t="inlineStr">
+      <c r="E10" s="38" t="inlineStr">
         <is>
           <t>per FP conv.</t>
         </is>
       </c>
-      <c r="F10" s="40">
+      <c r="F10" s="41">
         <f>Assumptions!$B$5</f>
         <v/>
       </c>
-      <c r="G10" s="38">
+      <c r="G10" s="39">
         <f>C10*F10</f>
         <v/>
       </c>
-      <c r="H10" s="38">
+      <c r="H10" s="39">
         <f>C10*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="I10" s="39">
+      <c r="I10" s="40">
         <f>D10*G10</f>
         <v/>
       </c>
-      <c r="J10" s="39">
+      <c r="J10" s="40">
         <f>I10*12</f>
         <v/>
       </c>
-      <c r="K10" s="39">
+      <c r="K10" s="40">
         <f>I10/G10</f>
         <v/>
       </c>
-      <c r="L10" s="41">
+      <c r="L10" s="42">
         <f>I10/H10</f>
         <v/>
       </c>
-      <c r="M10" s="42">
+      <c r="M10" s="43">
         <f>L10/Assumptions!$B$8-1</f>
         <v/>
       </c>
-      <c r="N10" s="43">
-        <f>Assumptions!$B$13</f>
-        <v/>
-      </c>
-      <c r="O10" s="43">
-        <f>Assumptions!$B$14</f>
-        <v/>
-      </c>
-      <c r="P10" s="43">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15)</f>
-        <v/>
-      </c>
-      <c r="Q10" s="44">
+      <c r="N10" s="44">
+        <f>Assumptions!$B$13*Assumptions!$B$19</f>
+        <v/>
+      </c>
+      <c r="O10" s="44">
+        <f>Assumptions!$B$14*Assumptions!$B$19</f>
+        <v/>
+      </c>
+      <c r="P10" s="44">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19)</f>
+        <v/>
+      </c>
+      <c r="Q10" s="45">
         <f>N10/K10</f>
         <v/>
       </c>
-      <c r="R10" s="44">
+      <c r="R10" s="45">
         <f>O10/K10</f>
         <v/>
       </c>
-      <c r="S10" s="45">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15/K10)</f>
-        <v/>
-      </c>
-      <c r="T10" s="39">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*G10)</f>
-        <v/>
-      </c>
-      <c r="U10" s="39">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*G10*12)</f>
-        <v/>
-      </c>
-      <c r="V10" s="46">
-        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15-K10)</f>
-        <v/>
-      </c>
-      <c r="W10" s="47">
-        <f>IF(Assumptions!$B$15="","n.a.",(Assumptions!$B$15-K10)*G10*12)</f>
+      <c r="S10" s="46">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19/K10)</f>
+        <v/>
+      </c>
+      <c r="T10" s="40">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19*G10)</f>
+        <v/>
+      </c>
+      <c r="U10" s="40">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19*G10*12)</f>
+        <v/>
+      </c>
+      <c r="V10" s="47">
+        <f>IF(Assumptions!$B$15="","n.a.",Assumptions!$B$15*Assumptions!$B$19-K10)</f>
+        <v/>
+      </c>
+      <c r="W10" s="48">
+        <f>IF(Assumptions!$B$15="","n.a.",(Assumptions!$B$15*Assumptions!$B$19-K10)*G10*12)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="48" t="inlineStr">
+      <c r="A12" s="49" t="inlineStr">
         <is>
           <t>• HEADLINE: at 36-mo LTV (~$164.51/shop) the funnel is LTV-negative at every payout — LTV:CAC = LTV ÷ payout = 0.66 ($250) · 0.55 ($300) · 0.47 ($350); iCAC runs 21–69% over the $267 target.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="48" t="inlineStr">
+      <c r="A13" s="49" t="inlineStr">
         <is>
           <t>• BUT the proposal still wins on both structural axes vs the 3-mo status quo: CVR 31% → 49%, and 1-mo-era per-shop LTV is higher ($93.35 vs $74.87 @12mo).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="48" t="inlineStr">
+      <c r="A14" s="49" t="inlineStr">
         <is>
           <t>• iGA (incremental gross adds) = paid trials × IAF; iCAC = monthly spend ÷ iGA = payout × CVR ÷ IAF. LTV:CAC uses cost per FP shop (= payout for the new model).</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="48" t="inlineStr">
+      <c r="A15" s="49" t="inlineStr">
         <is>
           <t>• Current state uses 3-mo-era LTV; @36mo not yet aged → shows 'n.a.'. New scenarios use 1-mo-era (go-forward) LTV. All-US.</t>
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="49" t="inlineStr">
+        <is>
+          <t>• LTV-DROP CONCERN (lead): go-forward LTV here is the 1-mo-era observed value, which ALREADY includes lower-intent marginal converters. To stress-test further, set 'LTV realization factor' on Assumptions (e.g. 80%) — see the LTV sensitivity tab for the full grid and breakeven.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A13:W13"/>
     <mergeCell ref="A14:W14"/>
     <mergeCell ref="N2:S2"/>
@@ -1923,6 +1970,7 @@
     <mergeCell ref="A12:W12"/>
     <mergeCell ref="I2:M2"/>
     <mergeCell ref="T2:W2"/>
+    <mergeCell ref="A16:W16"/>
     <mergeCell ref="F2:H2"/>
     <mergeCell ref="A15:W15"/>
   </mergeCells>
@@ -1964,32 +2012,32 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="49" t="inlineStr">
+      <c r="A4" s="50" t="inlineStr">
         <is>
           <t>iCAC ($)</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n"/>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="16" t="n"/>
+      <c r="B4" s="17" t="n"/>
+      <c r="C4" s="17" t="n"/>
+      <c r="D4" s="17" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="50" t="inlineStr">
+      <c r="A5" s="51" t="inlineStr">
         <is>
           <t>Payout \ IAF</t>
         </is>
       </c>
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>IAF 0.38 (low)</t>
         </is>
       </c>
-      <c r="C5" s="23" t="inlineStr">
+      <c r="C5" s="24" t="inlineStr">
         <is>
           <t>IAF 0.60 (mid)</t>
         </is>
       </c>
-      <c r="D5" s="23" t="inlineStr">
+      <c r="D5" s="24" t="inlineStr">
         <is>
           <t>IAF 0.75 (high)</t>
         </is>
@@ -2002,15 +2050,15 @@
         </is>
       </c>
       <c r="B6" s="10">
-        <f>Assumptions!$B$10*Assumptions!$B$5/Assumptions!$B$19</f>
+        <f>Assumptions!$B$10*Assumptions!$B$5/Assumptions!$B$20</f>
         <v/>
       </c>
       <c r="C6" s="10">
-        <f>Assumptions!$B$10*Assumptions!$B$5/Assumptions!$B$20</f>
+        <f>Assumptions!$B$10*Assumptions!$B$5/Assumptions!$B$21</f>
         <v/>
       </c>
       <c r="D6" s="10">
-        <f>Assumptions!$B$10*Assumptions!$B$5/Assumptions!$B$21</f>
+        <f>Assumptions!$B$10*Assumptions!$B$5/Assumptions!$B$22</f>
         <v/>
       </c>
     </row>
@@ -2021,15 +2069,15 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>Assumptions!$B$11*Assumptions!$B$5/Assumptions!$B$19</f>
+        <f>Assumptions!$B$11*Assumptions!$B$5/Assumptions!$B$20</f>
         <v/>
       </c>
       <c r="C7" s="10">
-        <f>Assumptions!$B$11*Assumptions!$B$5/Assumptions!$B$20</f>
+        <f>Assumptions!$B$11*Assumptions!$B$5/Assumptions!$B$21</f>
         <v/>
       </c>
       <c r="D7" s="10">
-        <f>Assumptions!$B$11*Assumptions!$B$5/Assumptions!$B$21</f>
+        <f>Assumptions!$B$11*Assumptions!$B$5/Assumptions!$B$22</f>
         <v/>
       </c>
     </row>
@@ -2040,45 +2088,45 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>Assumptions!$B$12*Assumptions!$B$5/Assumptions!$B$19</f>
+        <f>Assumptions!$B$12*Assumptions!$B$5/Assumptions!$B$20</f>
         <v/>
       </c>
       <c r="C8" s="10">
-        <f>Assumptions!$B$12*Assumptions!$B$5/Assumptions!$B$20</f>
+        <f>Assumptions!$B$12*Assumptions!$B$5/Assumptions!$B$21</f>
         <v/>
       </c>
       <c r="D8" s="10">
-        <f>Assumptions!$B$12*Assumptions!$B$5/Assumptions!$B$21</f>
+        <f>Assumptions!$B$12*Assumptions!$B$5/Assumptions!$B$22</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="51" t="inlineStr">
+      <c r="A11" s="52" t="inlineStr">
         <is>
           <t>iCAC vs $267 target</t>
         </is>
       </c>
-      <c r="B11" s="18" t="n"/>
-      <c r="C11" s="18" t="n"/>
-      <c r="D11" s="18" t="n"/>
+      <c r="B11" s="19" t="n"/>
+      <c r="C11" s="19" t="n"/>
+      <c r="D11" s="19" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="50" t="inlineStr">
+      <c r="A12" s="51" t="inlineStr">
         <is>
           <t>Payout \ IAF</t>
         </is>
       </c>
-      <c r="B12" s="23" t="inlineStr">
+      <c r="B12" s="24" t="inlineStr">
         <is>
           <t>IAF 0.38 (low)</t>
         </is>
       </c>
-      <c r="C12" s="23" t="inlineStr">
+      <c r="C12" s="24" t="inlineStr">
         <is>
           <t>IAF 0.60 (mid)</t>
         </is>
       </c>
-      <c r="D12" s="23" t="inlineStr">
+      <c r="D12" s="24" t="inlineStr">
         <is>
           <t>IAF 0.75 (high)</t>
         </is>
@@ -2090,16 +2138,16 @@
           <t>$250 / FP</t>
         </is>
       </c>
-      <c r="B13" s="52">
-        <f>(Assumptions!$B$10*Assumptions!$B$5/Assumptions!$B$19)/Assumptions!$B$8-1</f>
-        <v/>
-      </c>
-      <c r="C13" s="52">
+      <c r="B13" s="53">
         <f>(Assumptions!$B$10*Assumptions!$B$5/Assumptions!$B$20)/Assumptions!$B$8-1</f>
         <v/>
       </c>
-      <c r="D13" s="52">
+      <c r="C13" s="53">
         <f>(Assumptions!$B$10*Assumptions!$B$5/Assumptions!$B$21)/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+      <c r="D13" s="53">
+        <f>(Assumptions!$B$10*Assumptions!$B$5/Assumptions!$B$22)/Assumptions!$B$8-1</f>
         <v/>
       </c>
     </row>
@@ -2109,16 +2157,16 @@
           <t>$300 / FP</t>
         </is>
       </c>
-      <c r="B14" s="52">
-        <f>(Assumptions!$B$11*Assumptions!$B$5/Assumptions!$B$19)/Assumptions!$B$8-1</f>
-        <v/>
-      </c>
-      <c r="C14" s="52">
+      <c r="B14" s="53">
         <f>(Assumptions!$B$11*Assumptions!$B$5/Assumptions!$B$20)/Assumptions!$B$8-1</f>
         <v/>
       </c>
-      <c r="D14" s="52">
+      <c r="C14" s="53">
         <f>(Assumptions!$B$11*Assumptions!$B$5/Assumptions!$B$21)/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+      <c r="D14" s="53">
+        <f>(Assumptions!$B$11*Assumptions!$B$5/Assumptions!$B$22)/Assumptions!$B$8-1</f>
         <v/>
       </c>
     </row>
@@ -2128,16 +2176,16 @@
           <t>$350 / FP</t>
         </is>
       </c>
-      <c r="B15" s="52">
-        <f>(Assumptions!$B$12*Assumptions!$B$5/Assumptions!$B$19)/Assumptions!$B$8-1</f>
-        <v/>
-      </c>
-      <c r="C15" s="52">
+      <c r="B15" s="53">
         <f>(Assumptions!$B$12*Assumptions!$B$5/Assumptions!$B$20)/Assumptions!$B$8-1</f>
         <v/>
       </c>
-      <c r="D15" s="52">
+      <c r="C15" s="53">
         <f>(Assumptions!$B$12*Assumptions!$B$5/Assumptions!$B$21)/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+      <c r="D15" s="53">
+        <f>(Assumptions!$B$12*Assumptions!$B$5/Assumptions!$B$22)/Assumptions!$B$8-1</f>
         <v/>
       </c>
     </row>
@@ -2156,14 +2204,402 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A39"/>
+  <dimension ref="A1:F24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>LTV sensitivity — addressing 'LTV drops with a 1-month trial'</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>The lead's concern is marginal-converter dilution: a shorter trial converts more people (31%→49%), and the extra converters can be lower-LTV. The 1-mo-era LTV we use ($164.51 @36mo) already reflects that regime. Below: LTV:CAC and net contribution per shop @36mo as the go-forward LTV is haircut from 100% down to 60% of observed. BREAKEVEN (LTV:CAC = 1.0) requires LTV/shop = payout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="6">
+      <c r="A6" s="54" t="inlineStr">
+        <is>
+          <t>LTV:CAC @36mo  (= LTV × factor ÷ payout)</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="n"/>
+      <c r="C6" s="21" t="n"/>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="21" t="n"/>
+      <c r="F6" s="21" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="51" t="inlineStr">
+        <is>
+          <t>Payout \ LTV realization</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>130%</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>100% (observed)</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>85%</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>70%</t>
+        </is>
+      </c>
+      <c r="F7" s="24" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>$250 / FP</t>
+        </is>
+      </c>
+      <c r="B8" s="55">
+        <f>Assumptions!$B$15*1.3/Assumptions!$B$10</f>
+        <v/>
+      </c>
+      <c r="C8" s="56">
+        <f>Assumptions!$B$15*1.0/Assumptions!$B$10</f>
+        <v/>
+      </c>
+      <c r="D8" s="55">
+        <f>Assumptions!$B$15*0.85/Assumptions!$B$10</f>
+        <v/>
+      </c>
+      <c r="E8" s="55">
+        <f>Assumptions!$B$15*0.7/Assumptions!$B$10</f>
+        <v/>
+      </c>
+      <c r="F8" s="55">
+        <f>Assumptions!$B$15*0.6/Assumptions!$B$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>$300 / FP</t>
+        </is>
+      </c>
+      <c r="B9" s="55">
+        <f>Assumptions!$B$15*1.3/Assumptions!$B$11</f>
+        <v/>
+      </c>
+      <c r="C9" s="56">
+        <f>Assumptions!$B$15*1.0/Assumptions!$B$11</f>
+        <v/>
+      </c>
+      <c r="D9" s="55">
+        <f>Assumptions!$B$15*0.85/Assumptions!$B$11</f>
+        <v/>
+      </c>
+      <c r="E9" s="55">
+        <f>Assumptions!$B$15*0.7/Assumptions!$B$11</f>
+        <v/>
+      </c>
+      <c r="F9" s="55">
+        <f>Assumptions!$B$15*0.6/Assumptions!$B$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>$350 / FP</t>
+        </is>
+      </c>
+      <c r="B10" s="55">
+        <f>Assumptions!$B$15*1.3/Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="C10" s="56">
+        <f>Assumptions!$B$15*1.0/Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="D10" s="55">
+        <f>Assumptions!$B$15*0.85/Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="E10" s="55">
+        <f>Assumptions!$B$15*0.7/Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="F10" s="55">
+        <f>Assumptions!$B$15*0.6/Assumptions!$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="57" t="inlineStr">
+        <is>
+          <t>Net contribution / shop @36mo ($)</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="n"/>
+      <c r="C13" s="23" t="n"/>
+      <c r="D13" s="23" t="n"/>
+      <c r="E13" s="23" t="n"/>
+      <c r="F13" s="23" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="51" t="inlineStr">
+        <is>
+          <t>Payout \ LTV realization</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>130%</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t>100% (observed)</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>85%</t>
+        </is>
+      </c>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t>70%</t>
+        </is>
+      </c>
+      <c r="F14" s="24" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>$250 / FP</t>
+        </is>
+      </c>
+      <c r="B15" s="58">
+        <f>Assumptions!$B$15*1.3-Assumptions!$B$10</f>
+        <v/>
+      </c>
+      <c r="C15" s="59">
+        <f>Assumptions!$B$15*1.0-Assumptions!$B$10</f>
+        <v/>
+      </c>
+      <c r="D15" s="58">
+        <f>Assumptions!$B$15*0.85-Assumptions!$B$10</f>
+        <v/>
+      </c>
+      <c r="E15" s="58">
+        <f>Assumptions!$B$15*0.7-Assumptions!$B$10</f>
+        <v/>
+      </c>
+      <c r="F15" s="58">
+        <f>Assumptions!$B$15*0.6-Assumptions!$B$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>$300 / FP</t>
+        </is>
+      </c>
+      <c r="B16" s="58">
+        <f>Assumptions!$B$15*1.3-Assumptions!$B$11</f>
+        <v/>
+      </c>
+      <c r="C16" s="59">
+        <f>Assumptions!$B$15*1.0-Assumptions!$B$11</f>
+        <v/>
+      </c>
+      <c r="D16" s="58">
+        <f>Assumptions!$B$15*0.85-Assumptions!$B$11</f>
+        <v/>
+      </c>
+      <c r="E16" s="58">
+        <f>Assumptions!$B$15*0.7-Assumptions!$B$11</f>
+        <v/>
+      </c>
+      <c r="F16" s="58">
+        <f>Assumptions!$B$15*0.6-Assumptions!$B$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>$350 / FP</t>
+        </is>
+      </c>
+      <c r="B17" s="58">
+        <f>Assumptions!$B$15*1.3-Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="C17" s="59">
+        <f>Assumptions!$B$15*1.0-Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="D17" s="58">
+        <f>Assumptions!$B$15*0.85-Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="E17" s="58">
+        <f>Assumptions!$B$15*0.7-Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="F17" s="58">
+        <f>Assumptions!$B$15*0.6-Assumptions!$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="60" t="inlineStr">
+        <is>
+          <t>Breakeven LTV/shop needed (LTV:CAC = 1.0)  =  the payout itself:</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="n"/>
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="19" t="n"/>
+      <c r="E20" s="19" t="n"/>
+      <c r="F20" s="19" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="51" t="inlineStr">
+        <is>
+          <t>Payout</t>
+        </is>
+      </c>
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>Breakeven LTV</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>Observed LTV @36mo</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="inlineStr">
+        <is>
+          <t>× uplift needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>$250 / FP</t>
+        </is>
+      </c>
+      <c r="B22" s="10">
+        <f>Assumptions!$B$10</f>
+        <v/>
+      </c>
+      <c r="C22" s="11">
+        <f>Assumptions!$B$15</f>
+        <v/>
+      </c>
+      <c r="D22" s="55">
+        <f>Assumptions!$B$10/Assumptions!$B$15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>$300 / FP</t>
+        </is>
+      </c>
+      <c r="B23" s="10">
+        <f>Assumptions!$B$11</f>
+        <v/>
+      </c>
+      <c r="C23" s="11">
+        <f>Assumptions!$B$15</f>
+        <v/>
+      </c>
+      <c r="D23" s="55">
+        <f>Assumptions!$B$11/Assumptions!$B$15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>$350 / FP</t>
+        </is>
+      </c>
+      <c r="B24" s="10">
+        <f>Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="C24" s="11">
+        <f>Assumptions!$B$15</f>
+        <v/>
+      </c>
+      <c r="D24" s="55">
+        <f>Assumptions!$B$12/Assumptions!$B$15</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F4"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="105" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="53" t="inlineStr">
+      <c r="A1" s="61" t="inlineStr">
         <is>
           <t>How this workbook works</t>
         </is>
@@ -2173,7 +2609,7 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="54" t="inlineStr">
+      <c r="A3" s="62" t="inlineStr">
         <is>
           <t>PURPOSE</t>
         </is>
@@ -2204,7 +2640,7 @@
       <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="54" t="inlineStr">
+      <c r="A8" s="62" t="inlineStr">
         <is>
           <t>TABS</t>
         </is>
@@ -2232,176 +2668,221 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  LTV sensitivity  – LTV:CAC &amp; net contribution as go-forward LTV is haircut 130%→60% of observed, plus breakeven.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="54" t="inlineStr">
+      <c r="A13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="62" t="inlineStr">
         <is>
           <t>KEY FORMULAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  FP shops/mo    = paid trials × CVR</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  iGA/mo         = paid trials × IAF            (incremental gross adds)</t>
+          <t xml:space="preserve">  FP shops/mo    = paid trials × CVR</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Monthly spend  = payout × FP shops            (new model; current = $90 × paid trials)</t>
+          <t xml:space="preserve">  iGA/mo         = paid trials × IAF            (incremental gross adds)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cost/FP shop   = monthly spend / FP shops     (= payout for the new model)</t>
+          <t xml:space="preserve">  Monthly spend  = payout × FP shops            (new model; current = $90 × paid trials)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  iCAC           = monthly spend / iGA          (= payout × CVR / IAF)</t>
+          <t xml:space="preserve">  Cost/FP shop   = monthly spend / FP shops     (= payout for the new model)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t xml:space="preserve">  iCAC           = monthly spend / iGA          (= payout × CVR / IAF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t xml:space="preserve">  LTV:CAC        = LTV per shop / cost per FP shop</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" s="54" t="inlineStr">
+      <c r="A21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="62" t="inlineStr">
         <is>
           <t>VALIDATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  iCAC: $250→$322 · $300→$387 · $350→$451 (vs $267 target).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t xml:space="preserve">  iCAC: $250→$322 · $300→$387 · $350→$451 (vs $267 target).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t xml:space="preserve">  LTV:CAC @36mo: $250→0.66 · $300→0.55 · $350→0.47.   (matches River's Slack figures)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr"/>
-    </row>
     <row r="25">
-      <c r="A25" s="54" t="inlineStr">
+      <c r="A25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="62" t="inlineStr">
         <is>
           <t>LTV SOURCE</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  shopify-dw.marketing.shop_ltv_mart_predictions_with_forecast</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">  US · payback_channel_group = 'Affiliates' ·</t>
+          <t xml:space="preserve">  shopify-dw.marketing.shop_ltv_mart_predictions_with_forecast</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  per-shop = predicted_cumulative_total_profit_with_forecast / gross_adds_count_with_forecast</t>
+          <t xml:space="preserve">  US · payback_channel_group = 'Affiliates' ·</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">    1-mo era (Apr–Nov 2024): $93.35 / $130.12 / $164.51 @ 12/24/36mo   (go-forward)</t>
+          <t xml:space="preserve">  per-shop = predicted_cumulative_total_profit_with_forecast / gross_adds_count_with_forecast</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t xml:space="preserve">    1-mo era (Apr–Nov 2024): $93.35 / $130.12 / $164.51 @ 12/24/36mo   (go-forward)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t xml:space="preserve">    3-mo era (Feb–Dec 2025): $74.87 / $128.52 / n.a.    @ 12/24/36mo   (current state)</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-    </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>DEFAULTS APPLIED (per River's recommendation)</t>
-        </is>
-      </c>
+      <c r="A32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume unit = paid trials (49% applied directly to trials).</t>
+          <t>DEFAULTS APPLIED (per River's recommendation)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Volume unit = paid trials (49% applied directly to trials).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Headline horizon = 36 months. LTV era = 1-mo (go-forward). Geo = all-US. IAF = 0.38 (+ sensitivity tab).</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr"/>
-    </row>
     <row r="36">
-      <c r="A36" s="54" t="inlineStr">
-        <is>
-          <t>HEADLINE TAKEAWAY</t>
-        </is>
-      </c>
+      <c r="A36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  On a straight per-shop basis the funnel is LTV-negative at all three payouts (36-mo LTV ~$165 &lt; payout),</t>
+      <c r="A37" s="62" t="inlineStr">
+        <is>
+          <t>LEAD'S 'LTV DROPS WITH A 1-MO TRIAL' CONCERN — HOW IT'S HANDLED</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  and iCAC is 21–69% over target — i.e. higher payouts buy the SAME customers for more. The structural</t>
+          <t xml:space="preserve">  The go-forward LTV is the observed 1-mo-era value, which already blends in lower-intent marginal converters.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  An adjustable 'LTV realization factor' (Assumptions!B19, default 100%) lets you haircut it for extra caution,</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  and the LTV sensitivity tab shows the full grid + breakeven. Key point: breakeven LTV = the payout, so at $350</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  the shop would need ~2.1× its observed LTV just to break even — the conclusion holds across the whole haircut range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="62" t="inlineStr">
+        <is>
+          <t>HEADLINE TAKEAWAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  On a straight per-shop basis the funnel is LTV-negative at all three payouts (36-mo LTV ~$165 &lt; payout),</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  and iCAC is 21–69% over target — i.e. higher payouts buy the SAME customers for more. The structural</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t xml:space="preserve">  win is still real: compressing 3-mo → 1-mo lifts CVR (31%→49%) AND per-shop LTV ($75→$93 @12mo).</t>
         </is>

</xml_diff>

<commit_message>
Add all-markets rate card tab (1-mo rate = March rate - 25%)
Per-region rate card for Adrian Morrison (21 markets) with editable discount
lever (default 25%) applied to the March rate. iCAC/LTV:CAC/net columns use US
CVR/IAF/LTV as placeholders for non-US rows (flagged) pending market data.

Co-authored-by: johnkalis <johnkalis@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/analysis/adrian-morrison/adrian_morrison_1mo_trial_icac_ltv.xlsx
+++ b/analysis/adrian-morrison/adrian_morrison_1mo_trial_icac_ltv.xlsx
@@ -11,7 +11,8 @@
     <sheet name="Scenarios" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="IAF sensitivity" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="LTV sensitivity" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="README" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="All markets" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="README" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,7 +28,7 @@
     <numFmt numFmtId="167" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0;[Red]-&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +57,10 @@
     <font>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00B71C1C"/>
     </font>
   </fonts>
   <fills count="12">
@@ -142,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -311,6 +316,24 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2592,14 +2615,1043 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A46"/>
+  <dimension ref="A1:K30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Adrian Morrison — all-market rate card  (1-mo trial rate = March rate − 25%)</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Discount applied to the March rate (single lever — edit B2):</t>
+        </is>
+      </c>
+      <c r="E2" s="61" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Rate columns (Old / March / 1-mo) are market-specific. CVR, IAF and LTV/shop are US figures used as PLACEHOLDERS for non-US rows (only the US row is data-backed) — replace per market when available, then iCAC / LTV:CAC / net update automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Old rate ($)</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>March rate ($)</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="inlineStr">
+        <is>
+          <t>1-mo trial rate ($)</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>CVR</t>
+        </is>
+      </c>
+      <c r="F5" s="24" t="inlineStr">
+        <is>
+          <t>IAF</t>
+        </is>
+      </c>
+      <c r="G5" s="24" t="inlineStr">
+        <is>
+          <t>iCAC ($)</t>
+        </is>
+      </c>
+      <c r="H5" s="24" t="inlineStr">
+        <is>
+          <t>LTV/shop @36mo ($)</t>
+        </is>
+      </c>
+      <c r="I5" s="24" t="inlineStr">
+        <is>
+          <t>LTV:CAC</t>
+        </is>
+      </c>
+      <c r="J5" s="24" t="inlineStr">
+        <is>
+          <t>Net contrib/shop ($)</t>
+        </is>
+      </c>
+      <c r="K5" s="24" t="inlineStr">
+        <is>
+          <t>iCAC vs $267*</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="62" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="B6" s="40" t="n">
+        <v>225</v>
+      </c>
+      <c r="C6" s="40" t="n">
+        <v>75</v>
+      </c>
+      <c r="D6" s="63">
+        <f>C6*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F6" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G6" s="40">
+        <f>D6*E6/F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I6" s="46">
+        <f>H6/D6</f>
+        <v/>
+      </c>
+      <c r="J6" s="47">
+        <f>H6-D6</f>
+        <v/>
+      </c>
+      <c r="K6" s="43">
+        <f>G6/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="62" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="n">
+        <v>275</v>
+      </c>
+      <c r="C7" s="40" t="n">
+        <v>300</v>
+      </c>
+      <c r="D7" s="63">
+        <f>C7*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F7" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G7" s="40">
+        <f>D7*E7/F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I7" s="46">
+        <f>H7/D7</f>
+        <v/>
+      </c>
+      <c r="J7" s="47">
+        <f>H7-D7</f>
+        <v/>
+      </c>
+      <c r="K7" s="43">
+        <f>G7/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="62" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B8" s="40" t="n">
+        <v>275</v>
+      </c>
+      <c r="C8" s="40" t="n">
+        <v>350</v>
+      </c>
+      <c r="D8" s="63">
+        <f>C8*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E8" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F8" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G8" s="40">
+        <f>D8*E8/F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I8" s="46">
+        <f>H8/D8</f>
+        <v/>
+      </c>
+      <c r="J8" s="47">
+        <f>H8-D8</f>
+        <v/>
+      </c>
+      <c r="K8" s="43">
+        <f>G8/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="62" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B9" s="40" t="n">
+        <v>275</v>
+      </c>
+      <c r="C9" s="40" t="n">
+        <v>300</v>
+      </c>
+      <c r="D9" s="63">
+        <f>C9*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F9" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G9" s="40">
+        <f>D9*E9/F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I9" s="46">
+        <f>H9/D9</f>
+        <v/>
+      </c>
+      <c r="J9" s="47">
+        <f>H9-D9</f>
+        <v/>
+      </c>
+      <c r="K9" s="43">
+        <f>G9/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="62" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="B10" s="40" t="n">
+        <v>225</v>
+      </c>
+      <c r="C10" s="40" t="n">
+        <v>350</v>
+      </c>
+      <c r="D10" s="63">
+        <f>C10*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E10" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F10" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G10" s="40">
+        <f>D10*E10/F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I10" s="46">
+        <f>H10/D10</f>
+        <v/>
+      </c>
+      <c r="J10" s="47">
+        <f>H10-D10</f>
+        <v/>
+      </c>
+      <c r="K10" s="43">
+        <f>G10/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="62" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B11" s="40" t="n">
+        <v>225</v>
+      </c>
+      <c r="C11" s="40" t="n">
+        <v>350</v>
+      </c>
+      <c r="D11" s="63">
+        <f>C11*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F11" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G11" s="40">
+        <f>D11*E11/F11</f>
+        <v/>
+      </c>
+      <c r="H11" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I11" s="46">
+        <f>H11/D11</f>
+        <v/>
+      </c>
+      <c r="J11" s="47">
+        <f>H11-D11</f>
+        <v/>
+      </c>
+      <c r="K11" s="43">
+        <f>G11/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="62" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B12" s="40" t="n">
+        <v>275</v>
+      </c>
+      <c r="C12" s="40" t="n">
+        <v>350</v>
+      </c>
+      <c r="D12" s="63">
+        <f>C12*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F12" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G12" s="40">
+        <f>D12*E12/F12</f>
+        <v/>
+      </c>
+      <c r="H12" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I12" s="46">
+        <f>H12/D12</f>
+        <v/>
+      </c>
+      <c r="J12" s="47">
+        <f>H12-D12</f>
+        <v/>
+      </c>
+      <c r="K12" s="43">
+        <f>G12/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="62" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="B13" s="40" t="n">
+        <v>225</v>
+      </c>
+      <c r="C13" s="40" t="n">
+        <v>300</v>
+      </c>
+      <c r="D13" s="63">
+        <f>C13*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E13" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F13" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G13" s="40">
+        <f>D13*E13/F13</f>
+        <v/>
+      </c>
+      <c r="H13" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I13" s="46">
+        <f>H13/D13</f>
+        <v/>
+      </c>
+      <c r="J13" s="47">
+        <f>H13-D13</f>
+        <v/>
+      </c>
+      <c r="K13" s="43">
+        <f>G13/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="62" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B14" s="40" t="n">
+        <v>50</v>
+      </c>
+      <c r="C14" s="40" t="n">
+        <v>25</v>
+      </c>
+      <c r="D14" s="63">
+        <f>C14*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E14" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F14" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G14" s="40">
+        <f>D14*E14/F14</f>
+        <v/>
+      </c>
+      <c r="H14" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I14" s="46">
+        <f>H14/D14</f>
+        <v/>
+      </c>
+      <c r="J14" s="47">
+        <f>H14-D14</f>
+        <v/>
+      </c>
+      <c r="K14" s="43">
+        <f>G14/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="62" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="B15" s="40" t="n">
+        <v>275</v>
+      </c>
+      <c r="C15" s="40" t="n">
+        <v>300</v>
+      </c>
+      <c r="D15" s="63">
+        <f>C15*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E15" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F15" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G15" s="40">
+        <f>D15*E15/F15</f>
+        <v/>
+      </c>
+      <c r="H15" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I15" s="46">
+        <f>H15/D15</f>
+        <v/>
+      </c>
+      <c r="J15" s="47">
+        <f>H15-D15</f>
+        <v/>
+      </c>
+      <c r="K15" s="43">
+        <f>G15/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="62" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="B16" s="40" t="n">
+        <v>225</v>
+      </c>
+      <c r="C16" s="40" t="n">
+        <v>300</v>
+      </c>
+      <c r="D16" s="63">
+        <f>C16*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F16" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G16" s="40">
+        <f>D16*E16/F16</f>
+        <v/>
+      </c>
+      <c r="H16" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I16" s="46">
+        <f>H16/D16</f>
+        <v/>
+      </c>
+      <c r="J16" s="47">
+        <f>H16-D16</f>
+        <v/>
+      </c>
+      <c r="K16" s="43">
+        <f>G16/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="62" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="B17" s="40" t="n">
+        <v>275</v>
+      </c>
+      <c r="C17" s="40" t="n">
+        <v>300</v>
+      </c>
+      <c r="D17" s="63">
+        <f>C17*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E17" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F17" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G17" s="40">
+        <f>D17*E17/F17</f>
+        <v/>
+      </c>
+      <c r="H17" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I17" s="46">
+        <f>H17/D17</f>
+        <v/>
+      </c>
+      <c r="J17" s="47">
+        <f>H17-D17</f>
+        <v/>
+      </c>
+      <c r="K17" s="43">
+        <f>G17/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="62" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
+      <c r="B18" s="40" t="n">
+        <v>50</v>
+      </c>
+      <c r="C18" s="40" t="n">
+        <v>50</v>
+      </c>
+      <c r="D18" s="63">
+        <f>C18*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E18" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F18" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G18" s="40">
+        <f>D18*E18/F18</f>
+        <v/>
+      </c>
+      <c r="H18" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I18" s="46">
+        <f>H18/D18</f>
+        <v/>
+      </c>
+      <c r="J18" s="47">
+        <f>H18-D18</f>
+        <v/>
+      </c>
+      <c r="K18" s="43">
+        <f>G18/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="62" t="inlineStr">
+        <is>
+          <t>Middle East</t>
+        </is>
+      </c>
+      <c r="B19" s="40" t="n">
+        <v>225</v>
+      </c>
+      <c r="C19" s="40" t="n">
+        <v>200</v>
+      </c>
+      <c r="D19" s="63">
+        <f>C19*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E19" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F19" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G19" s="40">
+        <f>D19*E19/F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I19" s="46">
+        <f>H19/D19</f>
+        <v/>
+      </c>
+      <c r="J19" s="47">
+        <f>H19-D19</f>
+        <v/>
+      </c>
+      <c r="K19" s="43">
+        <f>G19/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="62" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="B20" s="40" t="n">
+        <v>225</v>
+      </c>
+      <c r="C20" s="40" t="n">
+        <v>300</v>
+      </c>
+      <c r="D20" s="63">
+        <f>C20*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E20" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F20" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G20" s="40">
+        <f>D20*E20/F20</f>
+        <v/>
+      </c>
+      <c r="H20" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I20" s="46">
+        <f>H20/D20</f>
+        <v/>
+      </c>
+      <c r="J20" s="47">
+        <f>H20-D20</f>
+        <v/>
+      </c>
+      <c r="K20" s="43">
+        <f>G20/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="62" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="B21" s="40" t="n">
+        <v>275</v>
+      </c>
+      <c r="C21" s="40" t="n">
+        <v>300</v>
+      </c>
+      <c r="D21" s="63">
+        <f>C21*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E21" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F21" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G21" s="40">
+        <f>D21*E21/F21</f>
+        <v/>
+      </c>
+      <c r="H21" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I21" s="46">
+        <f>H21/D21</f>
+        <v/>
+      </c>
+      <c r="J21" s="47">
+        <f>H21-D21</f>
+        <v/>
+      </c>
+      <c r="K21" s="43">
+        <f>G21/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="62" t="inlineStr">
+        <is>
+          <t>Rest of Asia</t>
+        </is>
+      </c>
+      <c r="B22" s="40" t="n">
+        <v>225</v>
+      </c>
+      <c r="C22" s="40" t="n">
+        <v>300</v>
+      </c>
+      <c r="D22" s="63">
+        <f>C22*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F22" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G22" s="40">
+        <f>D22*E22/F22</f>
+        <v/>
+      </c>
+      <c r="H22" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I22" s="46">
+        <f>H22/D22</f>
+        <v/>
+      </c>
+      <c r="J22" s="47">
+        <f>H22-D22</f>
+        <v/>
+      </c>
+      <c r="K22" s="43">
+        <f>G22/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="62" t="inlineStr">
+        <is>
+          <t>Rest of Europe</t>
+        </is>
+      </c>
+      <c r="B23" s="40" t="n">
+        <v>225</v>
+      </c>
+      <c r="C23" s="40" t="n">
+        <v>350</v>
+      </c>
+      <c r="D23" s="63">
+        <f>C23*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E23" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F23" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G23" s="40">
+        <f>D23*E23/F23</f>
+        <v/>
+      </c>
+      <c r="H23" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I23" s="46">
+        <f>H23/D23</f>
+        <v/>
+      </c>
+      <c r="J23" s="47">
+        <f>H23-D23</f>
+        <v/>
+      </c>
+      <c r="K23" s="43">
+        <f>G23/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="62" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="B24" s="40" t="n">
+        <v>275</v>
+      </c>
+      <c r="C24" s="40" t="n">
+        <v>300</v>
+      </c>
+      <c r="D24" s="63">
+        <f>C24*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E24" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F24" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G24" s="40">
+        <f>D24*E24/F24</f>
+        <v/>
+      </c>
+      <c r="H24" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I24" s="46">
+        <f>H24/D24</f>
+        <v/>
+      </c>
+      <c r="J24" s="47">
+        <f>H24-D24</f>
+        <v/>
+      </c>
+      <c r="K24" s="43">
+        <f>G24/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="62" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="B25" s="40" t="n">
+        <v>275</v>
+      </c>
+      <c r="C25" s="40" t="n">
+        <v>350</v>
+      </c>
+      <c r="D25" s="63">
+        <f>C25*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E25" s="13" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F25" s="64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G25" s="40">
+        <f>D25*E25/F25</f>
+        <v/>
+      </c>
+      <c r="H25" s="12" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I25" s="46">
+        <f>H25/D25</f>
+        <v/>
+      </c>
+      <c r="J25" s="47">
+        <f>H25-D25</f>
+        <v/>
+      </c>
+      <c r="K25" s="43">
+        <f>G25/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="25" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B26" s="28" t="n">
+        <v>275</v>
+      </c>
+      <c r="C26" s="28" t="n">
+        <v>350</v>
+      </c>
+      <c r="D26" s="65">
+        <f>C26*(1-'All markets'!$E$2)</f>
+        <v/>
+      </c>
+      <c r="E26" s="29" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F26" s="66" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G26" s="28">
+        <f>D26*E26/F26</f>
+        <v/>
+      </c>
+      <c r="H26" s="32" t="n">
+        <v>164.51</v>
+      </c>
+      <c r="I26" s="34">
+        <f>H26/D26</f>
+        <v/>
+      </c>
+      <c r="J26" s="35">
+        <f>H26-D26</f>
+        <v/>
+      </c>
+      <c r="K26" s="31">
+        <f>G26/Assumptions!$B$8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="49" t="inlineStr">
+        <is>
+          <t>• * iCAC vs $267 uses the US target as a reference only; market-specific iCAC targets differ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="49" t="inlineStr">
+        <is>
+          <t>• 1-mo trial rate = March rate × (1 − 25%). US: $350 → $262.50; UK/Canada/Rest of Europe → $262.50; most others ($300 March) → $225.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="49" t="inlineStr">
+        <is>
+          <t>• Shayna's UK/CA scale point: those markets carry the top $350 March rate, so they hold the most absolute room (→ $262.50).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A30:K30"/>
+    <mergeCell ref="A29:K29"/>
+    <mergeCell ref="A28:K28"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="105" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="61" t="inlineStr">
+      <c r="A1" s="67" t="inlineStr">
         <is>
           <t>How this workbook works</t>
         </is>
@@ -2609,7 +3661,7 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="62" t="inlineStr">
+      <c r="A3" s="68" t="inlineStr">
         <is>
           <t>PURPOSE</t>
         </is>
@@ -2640,7 +3692,7 @@
       <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="62" t="inlineStr">
+      <c r="A8" s="68" t="inlineStr">
         <is>
           <t>TABS</t>
         </is>
@@ -2675,214 +3727,221 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  All markets      – per-region rate card: 1-mo trial rate = March rate − 25%, with iCAC/LTV:CAC (US placeholders off-US).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="62" t="inlineStr">
+      <c r="A14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="68" t="inlineStr">
         <is>
           <t>KEY FORMULAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  FP shops/mo    = paid trials × CVR</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  iGA/mo         = paid trials × IAF            (incremental gross adds)</t>
+          <t xml:space="preserve">  FP shops/mo    = paid trials × CVR</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Monthly spend  = payout × FP shops            (new model; current = $90 × paid trials)</t>
+          <t xml:space="preserve">  iGA/mo         = paid trials × IAF            (incremental gross adds)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cost/FP shop   = monthly spend / FP shops     (= payout for the new model)</t>
+          <t xml:space="preserve">  Monthly spend  = payout × FP shops            (new model; current = $90 × paid trials)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  iCAC           = monthly spend / iGA          (= payout × CVR / IAF)</t>
+          <t xml:space="preserve">  Cost/FP shop   = monthly spend / FP shops     (= payout for the new model)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t xml:space="preserve">  iCAC           = monthly spend / iGA          (= payout × CVR / IAF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t xml:space="preserve">  LTV:CAC        = LTV per shop / cost per FP shop</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-    </row>
     <row r="22">
-      <c r="A22" s="62" t="inlineStr">
+      <c r="A22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="68" t="inlineStr">
         <is>
           <t>VALIDATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  iCAC: $250→$322 · $300→$387 · $350→$451 (vs $267 target).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t xml:space="preserve">  iCAC: $250→$322 · $300→$387 · $350→$451 (vs $267 target).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t xml:space="preserve">  LTV:CAC @36mo: $250→0.66 · $300→0.55 · $350→0.47.   (matches River's Slack figures)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-    </row>
     <row r="26">
-      <c r="A26" s="62" t="inlineStr">
+      <c r="A26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="68" t="inlineStr">
         <is>
           <t>LTV SOURCE</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  shopify-dw.marketing.shop_ltv_mart_predictions_with_forecast</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  US · payback_channel_group = 'Affiliates' ·</t>
+          <t xml:space="preserve">  shopify-dw.marketing.shop_ltv_mart_predictions_with_forecast</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  per-shop = predicted_cumulative_total_profit_with_forecast / gross_adds_count_with_forecast</t>
+          <t xml:space="preserve">  US · payback_channel_group = 'Affiliates' ·</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">    1-mo era (Apr–Nov 2024): $93.35 / $130.12 / $164.51 @ 12/24/36mo   (go-forward)</t>
+          <t xml:space="preserve">  per-shop = predicted_cumulative_total_profit_with_forecast / gross_adds_count_with_forecast</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t xml:space="preserve">    1-mo era (Apr–Nov 2024): $93.35 / $130.12 / $164.51 @ 12/24/36mo   (go-forward)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t xml:space="preserve">    3-mo era (Feb–Dec 2025): $74.87 / $128.52 / n.a.    @ 12/24/36mo   (current state)</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr"/>
-    </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>DEFAULTS APPLIED (per River's recommendation)</t>
-        </is>
-      </c>
+      <c r="A33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Volume unit = paid trials (49% applied directly to trials).</t>
+          <t>DEFAULTS APPLIED (per River's recommendation)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Volume unit = paid trials (49% applied directly to trials).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Headline horizon = 36 months. LTV era = 1-mo (go-forward). Geo = all-US. IAF = 0.38 (+ sensitivity tab).</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr"/>
-    </row>
     <row r="37">
-      <c r="A37" s="62" t="inlineStr">
+      <c r="A37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="68" t="inlineStr">
         <is>
           <t>LEAD'S 'LTV DROPS WITH A 1-MO TRIAL' CONCERN — HOW IT'S HANDLED</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  The go-forward LTV is the observed 1-mo-era value, which already blends in lower-intent marginal converters.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  An adjustable 'LTV realization factor' (Assumptions!B19, default 100%) lets you haircut it for extra caution,</t>
+          <t xml:space="preserve">  The go-forward LTV is the observed 1-mo-era value, which already blends in lower-intent marginal converters.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">  and the LTV sensitivity tab shows the full grid + breakeven. Key point: breakeven LTV = the payout, so at $350</t>
+          <t xml:space="preserve">  An adjustable 'LTV realization factor' (Assumptions!B19, default 100%) lets you haircut it for extra caution,</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t xml:space="preserve">  and the LTV sensitivity tab shows the full grid + breakeven. Key point: breakeven LTV = the payout, so at $350</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t xml:space="preserve">  the shop would need ~2.1× its observed LTV just to break even — the conclusion holds across the whole haircut range.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr"/>
-    </row>
     <row r="43">
-      <c r="A43" s="62" t="inlineStr">
+      <c r="A43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="68" t="inlineStr">
         <is>
           <t>HEADLINE TAKEAWAY</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  On a straight per-shop basis the funnel is LTV-negative at all three payouts (36-mo LTV ~$165 &lt; payout),</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">  and iCAC is 21–69% over target — i.e. higher payouts buy the SAME customers for more. The structural</t>
+          <t xml:space="preserve">  On a straight per-shop basis the funnel is LTV-negative at all three payouts (36-mo LTV ~$165 &lt; payout),</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  and iCAC is 21–69% over target — i.e. higher payouts buy the SAME customers for more. The structural</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t xml:space="preserve">  win is still real: compressing 3-mo → 1-mo lifts CVR (31%→49%) AND per-shop LTV ($75→$93 @12mo).</t>
         </is>

</xml_diff>